<commit_message>
establecimientos sin contar solo terapia intensiva
</commit_message>
<xml_diff>
--- a/TablasAnalisis/Cambios_en_la_edad_de_las_madres_con_porcentajes.xlsx
+++ b/TablasAnalisis/Cambios_en_la_edad_de_las_madres_con_porcentajes.xlsx
@@ -665,14 +665,14 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TIERRA DEL FUEGO</t>
+          <t>MENDOZA</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>12.9</v>
+        <v>15.57</v>
       </c>
       <c r="C16" t="n">
-        <v>4.81</v>
+        <v>7.48</v>
       </c>
       <c r="D16" t="n">
         <v>8.09</v>
@@ -681,14 +681,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MENDOZA</t>
+          <t>TIERRA DEL FUEGO</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>15.57</v>
+        <v>12.9</v>
       </c>
       <c r="C17" t="n">
-        <v>7.48</v>
+        <v>4.81</v>
       </c>
       <c r="D17" t="n">
         <v>8.09</v>

</xml_diff>

<commit_message>
agrego tasa fecundidad 2010
</commit_message>
<xml_diff>
--- a/TablasAnalisis/Cambios_en_la_edad_de_las_madres_con_porcentajes.xlsx
+++ b/TablasAnalisis/Cambios_en_la_edad_de_las_madres_con_porcentajes.xlsx
@@ -665,14 +665,14 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MENDOZA</t>
+          <t>TIERRA DEL FUEGO</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>15.57</v>
+        <v>12.9</v>
       </c>
       <c r="C16" t="n">
-        <v>7.48</v>
+        <v>4.81</v>
       </c>
       <c r="D16" t="n">
         <v>8.09</v>
@@ -681,14 +681,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TIERRA DEL FUEGO</t>
+          <t>MENDOZA</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>12.9</v>
+        <v>15.57</v>
       </c>
       <c r="C17" t="n">
-        <v>4.81</v>
+        <v>7.48</v>
       </c>
       <c r="D17" t="n">
         <v>8.09</v>

</xml_diff>

<commit_message>
tabla tasa 2010 vs tasa 2022
</commit_message>
<xml_diff>
--- a/TablasAnalisis/Cambios_en_la_edad_de_las_madres_con_porcentajes.xlsx
+++ b/TablasAnalisis/Cambios_en_la_edad_de_las_madres_con_porcentajes.xlsx
@@ -665,14 +665,14 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TIERRA DEL FUEGO</t>
+          <t>MENDOZA</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>12.9</v>
+        <v>15.57</v>
       </c>
       <c r="C16" t="n">
-        <v>4.81</v>
+        <v>7.48</v>
       </c>
       <c r="D16" t="n">
         <v>8.09</v>
@@ -681,14 +681,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>MENDOZA</t>
+          <t>TIERRA DEL FUEGO</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>15.57</v>
+        <v>12.9</v>
       </c>
       <c r="C17" t="n">
-        <v>7.48</v>
+        <v>4.81</v>
       </c>
       <c r="D17" t="n">
         <v>8.09</v>

</xml_diff>